<commit_message>
Backup working Central C&I system
</commit_message>
<xml_diff>
--- a/data/material_issue.xlsx
+++ b/data/material_issue.xlsx
@@ -16,12 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -51,10 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,137 +482,6 @@
           <t>Actual Return Date</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>MAT-20260807-001</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>46241</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Power Plant (3x130MW)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Positioner</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>9556602370</v>
-      </c>
-      <c r="I2" s="1" t="n">
-        <v>46241</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Avinash Ujjwal</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Issued</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MAT-20260807-001</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>46241</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Power Plant (3x130MW)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>EPSITA</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" s="1" t="n">
-        <v>46241</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Avinash Ujjwal</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Issued</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MAT-20260807-001</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46241</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Pellet Plant</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Actuator</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" s="2" t="n">
-        <v>46241</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Avinash Ujjwal</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Issued</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>